<commit_message>
loss dec ignored in contract code
</commit_message>
<xml_diff>
--- a/tests/test files/Bw0197222 claims.xlsx
+++ b/tests/test files/Bw0197222 claims.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tolia\Desktop\AI Projects\Claude projects all\Claude projects v3\Project\tests\test files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD62BB6-3846-4CD4-BA10-D7F213126CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685ADCFD-237A-46E2-9DC9-18A2406885B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="2940" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>Claim Number</t>
   </si>
@@ -109,7 +109,10 @@
     <t>CR007</t>
   </si>
   <si>
-    <t>BW0197322</t>
+    <t>Legal expense Claim</t>
+  </si>
+  <si>
+    <t>Loss Description</t>
   </si>
 </sst>
 </file>
@@ -374,7 +377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="11.5" customWidth="1"/>
@@ -384,7 +387,7 @@
     <col min="6" max="6" width="5.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -407,12 +410,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15">
+    <row r="3" spans="1:8" ht="15">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,8 +432,11 @@
       <c r="G3" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -457,8 +458,11 @@
       <c r="G4" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -481,7 +485,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -504,7 +508,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:8">
       <c r="C7" t="s">
         <v>16</v>
       </c>
@@ -518,7 +522,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>17</v>
       </c>

</xml_diff>